<commit_message>
Completely remove THS auto-injected transactions and preserve clean personal transactions only
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -654,147 +654,9 @@
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>10:00:00 28/8/2026</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Quỹ Đầu tư THS</v>
-      </c>
-      <c r="E12">
-        <v>11516551</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Tài khoản Quỹ Đầu tư</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Lợi nhuận cổ đông Thịnh (42.86%) - Tháng 8 2026 [THS Chrono Online]</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>10:00:00 28/7/2026</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Quỹ Đầu tư THS</v>
-      </c>
-      <c r="E13">
-        <v>11574522</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Tài khoản Quỹ Đầu tư</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Lợi nhuận cổ đông Thịnh (42.86%) - Tháng 7 2026 [THS Chrono Online]</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>10:00:00 28/6/2026</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Quỹ Đầu tư THS</v>
-      </c>
-      <c r="E14">
-        <v>14455246</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Tài khoản Quỹ Đầu tư</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Lợi nhuận cổ đông Thịnh (42.86%) - Tháng 6 2026 [THS Chrono Online]</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>10:00:00 28/5/2026</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Quỹ Đầu tư THS</v>
-      </c>
-      <c r="E15">
-        <v>13727124</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Tài khoản Quỹ Đầu tư</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Lợi nhuận cổ đông Thịnh (42.86%) - Tháng 5 2026 [THS Chrono Online]</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>10:00:00 28/4/2026</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Quỹ Đầu tư THS</v>
-      </c>
-      <c r="E16">
-        <v>20487143</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Tài khoản Quỹ Đầu tư</v>
-      </c>
-      <c r="G16" t="str">
-        <v>Lợi nhuận cổ đông Thịnh (42.86%) - Tháng 4 2026 [THS Chrono Online]</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>10:00:00 28/3/2026</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Quỹ Đầu tư THS</v>
-      </c>
-      <c r="E17">
-        <v>13040596</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Tài khoản Quỹ Đầu tư</v>
-      </c>
-      <c r="G17" t="str">
-        <v>Lợi nhuận cổ đông Thịnh (42.86%) - Tháng 3 2026 [THS Chrono Online]</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -966,7 +828,7 @@
         <v>investment</v>
       </c>
       <c r="D5">
-        <v>84801182</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reset all transactions, wipe Google Sheet and prepare fresh database for October 2026
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -399,264 +399,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>STT</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Thời gian</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Phân loại</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Khoản mục / Nguồn thu</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Số tiền (VNĐ)</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Ví thanh toán</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Ghi chú</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>15:30:00 11/9/2026</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Không xác định</v>
-      </c>
-      <c r="E2">
-        <v>4500000</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Thu nhập khác</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>11:20:00 11/9/2026</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Chi tiêu</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ăn uống &amp; Cà phê</v>
-      </c>
-      <c r="E3">
-        <v>104000</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Chi tiêu sinh hoạt</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>19:00:00 10/9/2026</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Chi tiêu</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Chi phí khác</v>
-      </c>
-      <c r="E4">
-        <v>50000</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Chi tiêu vặt</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>13:27:00 10/9/2026</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Chi tiêu</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Ăn uống &amp; Cà phê</v>
-      </c>
-      <c r="E5">
-        <v>50000</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G5" t="str">
-        <v>ăn sáng</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>13:14:00 10/9/2026</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Không xác định</v>
-      </c>
-      <c r="E6">
-        <v>1000000</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>15:48:00 9/9/2026</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Không xác định</v>
-      </c>
-      <c r="E7">
-        <v>3500000</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G7" t="str">
-        <v>PB</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>15:48:00 9/9/2026</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Chi tiêu</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Ăn uống &amp; Cà phê</v>
-      </c>
-      <c r="E8">
-        <v>200000</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G8" t="str">
-        <v>ăn sáng cùng na</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>08:10:00 4/9/2026</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Chi tiêu</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
-      </c>
-      <c r="E9">
-        <v>70000</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Đổ xăng</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>15:52:00 3/9/2026</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Chi tiêu</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
-      </c>
-      <c r="E10">
-        <v>280000</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Chi mua vé bus</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>15:50:00 3/9/2026</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Lương hàng tháng</v>
-      </c>
-      <c r="E11">
-        <v>18000000</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -786,7 +532,7 @@
         <v>bank</v>
       </c>
       <c r="D2">
-        <v>26246000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Support reading/writing to monthly tabs (thang 10, thang 11) and automatic next month tab creation
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -399,10 +399,149 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Thời gian</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Phân loại</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Khoản mục / Nguồn thu</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Số tiền (VNĐ)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Ví thanh toán</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Ghi chú</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Tiền đút lót</v>
+      </c>
+      <c r="E2">
+        <v>500000</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G2" t="str">
+        <v>PB</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Đầu tư THS</v>
+      </c>
+      <c r="E3">
+        <v>10411000</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Chi trả cổ phần tháng 9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Lương hàng tháng</v>
+      </c>
+      <c r="E4">
+        <v>18000000</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Nhận lương tháng 10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E5">
+        <v>280000</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Vé bus tháng 10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E6">
+        <v>90000</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Đổ xăng xe máy</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -532,7 +671,7 @@
         <v>bank</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>28041000</v>
       </c>
     </row>
     <row r="3">
@@ -546,7 +685,7 @@
         <v>cash</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Sync updated Google Sheet Month 10 layout to Web and Render
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -478,19 +478,19 @@
         <v>19:00:00 1/10/2026</v>
       </c>
       <c r="C4" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D4" t="str">
-        <v>Lương hàng tháng</v>
+        <v>Đi lại &amp; Xăng xe</v>
       </c>
       <c r="E4">
-        <v>18000000</v>
+        <v>90000</v>
       </c>
       <c r="F4" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G4" t="str">
-        <v>Nhận lương tháng 10</v>
+        <v>Đổ xăng xe máy</v>
       </c>
     </row>
     <row r="5">
@@ -513,7 +513,7 @@
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G5" t="str">
-        <v>Vé bus tháng 10</v>
+        <v>Vé xe bus</v>
       </c>
     </row>
     <row r="6">
@@ -524,19 +524,19 @@
         <v>19:00:00 1/10/2026</v>
       </c>
       <c r="C6" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D6" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
+        <v>Lương hàng tháng</v>
       </c>
       <c r="E6">
-        <v>90000</v>
+        <v>18000000</v>
       </c>
       <c r="F6" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G6" t="str">
-        <v>Đổ xăng xe máy</v>
+        <v>lương tháng 10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Categorize Tien dut lot under Khong xac dinh in income breakdown
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -429,22 +429,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>19:00:00 3/10/2026</v>
+        <v>19:00:00 1/10/2026</v>
       </c>
       <c r="C2" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D2" t="str">
-        <v>Tiền đút lót</v>
+        <v>Đi lại &amp; Xăng xe</v>
       </c>
       <c r="E2">
-        <v>500000</v>
+        <v>90000</v>
       </c>
       <c r="F2" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G2" t="str">
-        <v>PB</v>
+        <v>Đổ xăng xe máy</v>
       </c>
     </row>
     <row r="3">
@@ -458,16 +458,16 @@
         <v>Thu nhập</v>
       </c>
       <c r="D3" t="str">
-        <v>Đầu tư THS</v>
+        <v>Không xác định</v>
       </c>
       <c r="E3">
-        <v>10411000</v>
+        <v>500000</v>
       </c>
       <c r="F3" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
+        <v>Tiền mặt</v>
       </c>
       <c r="G3" t="str">
-        <v>Chi trả cổ phần tháng 9</v>
+        <v>PB (Tiền đút lót)</v>
       </c>
     </row>
     <row r="4">
@@ -475,22 +475,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>19:00:00 1/10/2026</v>
+        <v>19:00:00 3/10/2026</v>
       </c>
       <c r="C4" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D4" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
+        <v>Quỹ Đầu tư THS</v>
       </c>
       <c r="E4">
-        <v>90000</v>
+        <v>10411000</v>
       </c>
       <c r="F4" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G4" t="str">
-        <v>Đổ xăng xe máy</v>
+        <v>Chi trả cổ phần tháng 9</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Fix sync for transactions without date cell and ensure 100% match with Google Sheet
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,7 +429,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>19:00:00 1/10/2026</v>
+        <v>19:00:00 19/10/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Chi tiêu</v>
@@ -438,13 +438,13 @@
         <v>Đi lại &amp; Xăng xe</v>
       </c>
       <c r="E2">
-        <v>90000</v>
+        <v>600000</v>
       </c>
       <c r="F2" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G2" t="str">
-        <v>Đổ xăng xe máy</v>
+        <v>Tiền gửi xe</v>
       </c>
     </row>
     <row r="3">
@@ -452,22 +452,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>19:00:00 3/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C3" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D3" t="str">
-        <v>Không xác định</v>
+        <v>Nhà cửa &amp; Hóa đơn</v>
       </c>
       <c r="E3">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="F3" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G3" t="str">
-        <v>PB (Tiền đút lót)</v>
+        <v>Tiền đt</v>
       </c>
     </row>
     <row r="4">
@@ -475,22 +475,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>19:00:00 3/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C4" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D4" t="str">
-        <v>Quỹ Đầu tư THS</v>
+        <v>Ăn uống &amp; Cà phê</v>
       </c>
       <c r="E4">
-        <v>10411000</v>
+        <v>240000</v>
       </c>
       <c r="F4" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G4" t="str">
-        <v>Chi trả cổ phần tháng 9</v>
+        <v>Bún đậu</v>
       </c>
     </row>
     <row r="5">
@@ -498,22 +498,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>19:00:00 1/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D5" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
+        <v>Giải trí &amp; Du lịch</v>
       </c>
       <c r="E5">
-        <v>280000</v>
+        <v>170000</v>
       </c>
       <c r="F5" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G5" t="str">
-        <v>Vé xe bus</v>
+        <v>Xem xiếc</v>
       </c>
     </row>
     <row r="6">
@@ -521,27 +521,602 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>19:00:00 1/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Thu nhập</v>
       </c>
       <c r="D6" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E6">
+        <v>2000000</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>19:00:00 12/10/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Ăn uống &amp; Cà phê</v>
+      </c>
+      <c r="E7">
+        <v>105000</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Ăn tối và mua bông ngoáy tai</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>19:00:00 12/10/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E8">
+        <v>1500000</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>19:00:00 12/10/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E9">
+        <v>1500000</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>19:00:00 11/10/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Ăn uống &amp; Cà phê</v>
+      </c>
+      <c r="E10">
+        <v>100000</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Ăn sáng cùng na</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>19:00:00 10/10/2026</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Ăn uống &amp; Cà phê</v>
+      </c>
+      <c r="E11">
+        <v>35000</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Bmy ăn sáng cho na</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>19:00:00 10/10/2026</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Sức khỏe &amp; Y tế</v>
+      </c>
+      <c r="E12">
+        <v>780000</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>19:00:00 9/10/2026</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E13">
+        <v>2000000</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Pbi</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>19:00:00 9/10/2026</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E14">
+        <v>90000</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>19:00:00 9/10/2026</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Ăn uống &amp; Cà phê</v>
+      </c>
+      <c r="E15">
+        <v>40000</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>19:00:00 8/10/2026</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E16">
+        <v>2500000</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Pbi</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>19:00:00 7/10/2026</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E17">
+        <v>1000000</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Pb</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>19:00:00 7/10/2026</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Nhà cửa &amp; Hóa đơn</v>
+      </c>
+      <c r="E18">
+        <v>377000</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>19:00:00 7/10/2026</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Mua sắm &amp; Tiêu dùng</v>
+      </c>
+      <c r="E19">
+        <v>152000</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>19:00:00 7/10/2026</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E20">
+        <v>3500000</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Pbi</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>19:00:00 6/10/2026</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E21">
+        <v>1000000</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Đút lót</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>19:00:00 6/10/2026</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E22">
+        <v>1350000</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Công tác phí</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>19:00:00 5/10/2026</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Học tập &amp; Kỹ năng</v>
+      </c>
+      <c r="E23">
+        <v>144000</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Đỡ đàn của Na</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>19:00:00 4/10/2026</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Chi phí khác</v>
+      </c>
+      <c r="E24">
+        <v>600000</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Ăn sáng, sửa sân....</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E25">
+        <v>500000</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G25" t="str">
+        <v>PB (Tiền đút lót)</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Quỹ Đầu tư THS</v>
+      </c>
+      <c r="E26">
+        <v>10411000</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Chi trả cổ phần tháng 9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Mua sắm &amp; Tiêu dùng</v>
+      </c>
+      <c r="E27">
+        <v>500000</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Đi chợ</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>19:00:00 2/10/2026</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Ăn uống &amp; Cà phê</v>
+      </c>
+      <c r="E28">
+        <v>50000</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Mua đồ ăn vặt cho na ne</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E29">
+        <v>90000</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Đổ xăng xe máy</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E30">
+        <v>280000</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Vé xe bus</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D31" t="str">
         <v>Lương hàng tháng</v>
       </c>
-      <c r="E6">
+      <c r="E31">
         <v>18000000</v>
       </c>
-      <c r="F6" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="F31" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G31" t="str">
         <v>lương tháng 10</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G31"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -671,7 +1246,7 @@
         <v>bank</v>
       </c>
       <c r="D2">
-        <v>28041000</v>
+        <v>30858000</v>
       </c>
     </row>
     <row r="3">
@@ -685,7 +1260,7 @@
         <v>cash</v>
       </c>
       <c r="D3">
-        <v>500000</v>
+        <v>9850000</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Fix: use stable row-based ID for Sheet txs, full-replace on sync to prevent stale/duplicate data
</commit_message>
<xml_diff>
--- a/data/finance_records.xlsx
+++ b/data/finance_records.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -613,7 +613,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>19:00:00 11/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C10" t="str">
         <v>Chi tiêu</v>
@@ -622,13 +622,13 @@
         <v>Ăn uống &amp; Cà phê</v>
       </c>
       <c r="E10">
-        <v>100000</v>
+        <v>380000</v>
       </c>
       <c r="F10" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G10" t="str">
-        <v>Ăn sáng cùng na</v>
+        <v>Ăn trưa cùng ban</v>
       </c>
     </row>
     <row r="11">
@@ -636,22 +636,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>19:00:00 10/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C11" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D11" t="str">
-        <v>Ăn uống &amp; Cà phê</v>
+        <v>Không xác định</v>
       </c>
       <c r="E11">
-        <v>35000</v>
+        <v>500000</v>
       </c>
       <c r="F11" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G11" t="str">
-        <v>Bmy ăn sáng cho na</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -659,16 +659,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>19:00:00 10/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C12" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D12" t="str">
-        <v>Sức khỏe &amp; Y tế</v>
+        <v>Không xác định</v>
       </c>
       <c r="E12">
-        <v>780000</v>
+        <v>2000000</v>
       </c>
       <c r="F12" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
@@ -682,7 +682,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>19:00:00 9/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Thu nhập</v>
@@ -697,7 +697,7 @@
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G13" t="str">
-        <v>Pbi</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -705,7 +705,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>19:00:00 9/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Chi tiêu</v>
@@ -714,7 +714,7 @@
         <v>Đi lại &amp; Xăng xe</v>
       </c>
       <c r="E14">
-        <v>90000</v>
+        <v>270000</v>
       </c>
       <c r="F14" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
@@ -728,16 +728,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>19:00:00 9/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C15" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D15" t="str">
-        <v>Ăn uống &amp; Cà phê</v>
+        <v>Không xác định</v>
       </c>
       <c r="E15">
-        <v>40000</v>
+        <v>500000</v>
       </c>
       <c r="F15" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
@@ -751,7 +751,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>19:00:00 8/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Thu nhập</v>
@@ -760,13 +760,13 @@
         <v>Không xác định</v>
       </c>
       <c r="E16">
-        <v>2500000</v>
+        <v>500000</v>
       </c>
       <c r="F16" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G16" t="str">
-        <v>Pbi</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -774,22 +774,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>19:00:00 7/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C17" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D17" t="str">
-        <v>Không xác định</v>
+        <v>Ăn uống &amp; Cà phê</v>
       </c>
       <c r="E17">
-        <v>1000000</v>
+        <v>860000</v>
       </c>
       <c r="F17" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G17" t="str">
-        <v>Pb</v>
+        <v>Ăn mời BVAN</v>
       </c>
     </row>
     <row r="18">
@@ -797,22 +797,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>19:00:00 7/10/2026</v>
+        <v>19:00:00 12/10/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D18" t="str">
-        <v>Nhà cửa &amp; Hóa đơn</v>
+        <v>Học tập &amp; Kỹ năng</v>
       </c>
       <c r="E18">
-        <v>377000</v>
+        <v>2500000</v>
       </c>
       <c r="F18" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>Tiền học đan của na</v>
       </c>
     </row>
     <row r="19">
@@ -820,22 +820,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>19:00:00 7/10/2026</v>
+        <v>19:00:00 11/10/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D19" t="str">
-        <v>Mua sắm &amp; Tiêu dùng</v>
+        <v>Ăn uống &amp; Cà phê</v>
       </c>
       <c r="E19">
-        <v>152000</v>
+        <v>100000</v>
       </c>
       <c r="F19" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>Ăn sáng cùng na</v>
       </c>
     </row>
     <row r="20">
@@ -843,22 +843,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>19:00:00 7/10/2026</v>
+        <v>19:00:00 10/10/2026</v>
       </c>
       <c r="C20" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D20" t="str">
-        <v>Không xác định</v>
+        <v>Ăn uống &amp; Cà phê</v>
       </c>
       <c r="E20">
-        <v>3500000</v>
+        <v>35000</v>
       </c>
       <c r="F20" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G20" t="str">
-        <v>Pbi</v>
+        <v>Bmy ăn sáng cho na</v>
       </c>
     </row>
     <row r="21">
@@ -866,22 +866,22 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>19:00:00 6/10/2026</v>
+        <v>19:00:00 10/10/2026</v>
       </c>
       <c r="C21" t="str">
-        <v>Thu nhập</v>
+        <v>Chi tiêu</v>
       </c>
       <c r="D21" t="str">
-        <v>Không xác định</v>
+        <v>Sức khỏe &amp; Y tế</v>
       </c>
       <c r="E21">
-        <v>1000000</v>
+        <v>780000</v>
       </c>
       <c r="F21" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G21" t="str">
-        <v>Đút lót</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -889,7 +889,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>19:00:00 6/10/2026</v>
+        <v>19:00:00 9/10/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Thu nhập</v>
@@ -898,13 +898,13 @@
         <v>Không xác định</v>
       </c>
       <c r="E22">
-        <v>1350000</v>
+        <v>2000000</v>
       </c>
       <c r="F22" t="str">
-        <v>Tiền mặt</v>
+        <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G22" t="str">
-        <v>Công tác phí</v>
+        <v>Pbi</v>
       </c>
     </row>
     <row r="23">
@@ -912,22 +912,22 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>19:00:00 5/10/2026</v>
+        <v>19:00:00 9/10/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D23" t="str">
-        <v>Học tập &amp; Kỹ năng</v>
+        <v>Đi lại &amp; Xăng xe</v>
       </c>
       <c r="E23">
-        <v>144000</v>
+        <v>90000</v>
       </c>
       <c r="F23" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G23" t="str">
-        <v>Đỡ đàn của Na</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -935,22 +935,22 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>19:00:00 4/10/2026</v>
+        <v>19:00:00 9/10/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D24" t="str">
-        <v>Chi phí khác</v>
+        <v>Ăn uống &amp; Cà phê</v>
       </c>
       <c r="E24">
-        <v>600000</v>
+        <v>40000</v>
       </c>
       <c r="F24" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G24" t="str">
-        <v>Ăn sáng, sửa sân....</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -958,7 +958,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>19:00:00 3/10/2026</v>
+        <v>19:00:00 8/10/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Thu nhập</v>
@@ -967,13 +967,13 @@
         <v>Không xác định</v>
       </c>
       <c r="E25">
-        <v>500000</v>
+        <v>2500000</v>
       </c>
       <c r="F25" t="str">
         <v>Tiền mặt</v>
       </c>
       <c r="G25" t="str">
-        <v>PB (Tiền đút lót)</v>
+        <v>Pbi</v>
       </c>
     </row>
     <row r="26">
@@ -981,22 +981,22 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>19:00:00 3/10/2026</v>
+        <v>19:00:00 7/10/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Thu nhập</v>
       </c>
       <c r="D26" t="str">
-        <v>Quỹ Đầu tư THS</v>
+        <v>Không xác định</v>
       </c>
       <c r="E26">
-        <v>10411000</v>
+        <v>1000000</v>
       </c>
       <c r="F26" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
+        <v>Tiền mặt</v>
       </c>
       <c r="G26" t="str">
-        <v>Chi trả cổ phần tháng 9</v>
+        <v>Pb</v>
       </c>
     </row>
     <row r="27">
@@ -1004,22 +1004,22 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>19:00:00 3/10/2026</v>
+        <v>19:00:00 7/10/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D27" t="str">
-        <v>Mua sắm &amp; Tiêu dùng</v>
+        <v>Nhà cửa &amp; Hóa đơn</v>
       </c>
       <c r="E27">
-        <v>500000</v>
+        <v>377000</v>
       </c>
       <c r="F27" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G27" t="str">
-        <v>Đi chợ</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1027,22 +1027,22 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>19:00:00 2/10/2026</v>
+        <v>19:00:00 7/10/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Chi tiêu</v>
       </c>
       <c r="D28" t="str">
-        <v>Ăn uống &amp; Cà phê</v>
+        <v>Mua sắm &amp; Tiêu dùng</v>
       </c>
       <c r="E28">
-        <v>50000</v>
+        <v>152000</v>
       </c>
       <c r="F28" t="str">
         <v>Tài khoản Ngân hàng (Chính)</v>
       </c>
       <c r="G28" t="str">
-        <v>Mua đồ ăn vặt cho na ne</v>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1050,22 +1050,22 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>19:00:00 1/10/2026</v>
+        <v>19:00:00 7/10/2026</v>
       </c>
       <c r="C29" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D29" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
+        <v>Không xác định</v>
       </c>
       <c r="E29">
-        <v>90000</v>
+        <v>3500000</v>
       </c>
       <c r="F29" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
+        <v>Tiền mặt</v>
       </c>
       <c r="G29" t="str">
-        <v>Đổ xăng xe máy</v>
+        <v>Pbi</v>
       </c>
     </row>
     <row r="30">
@@ -1073,22 +1073,22 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>19:00:00 1/10/2026</v>
+        <v>19:00:00 6/10/2026</v>
       </c>
       <c r="C30" t="str">
-        <v>Chi tiêu</v>
+        <v>Thu nhập</v>
       </c>
       <c r="D30" t="str">
-        <v>Đi lại &amp; Xăng xe</v>
+        <v>Không xác định</v>
       </c>
       <c r="E30">
-        <v>280000</v>
+        <v>1000000</v>
       </c>
       <c r="F30" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
+        <v>Tiền mặt</v>
       </c>
       <c r="G30" t="str">
-        <v>Vé xe bus</v>
+        <v>Đút lót</v>
       </c>
     </row>
     <row r="31">
@@ -1096,27 +1096,234 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
+        <v>19:00:00 6/10/2026</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E31">
+        <v>1350000</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Công tác phí</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>19:00:00 5/10/2026</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Học tập &amp; Kỹ năng</v>
+      </c>
+      <c r="E32">
+        <v>144000</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Đỡ đàn của Na</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>19:00:00 4/10/2026</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Chi phí khác</v>
+      </c>
+      <c r="E33">
+        <v>600000</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Ăn sáng, sửa sân....</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Không xác định</v>
+      </c>
+      <c r="E34">
+        <v>500000</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Tiền mặt</v>
+      </c>
+      <c r="G34" t="str">
+        <v>PB (Tiền đút lót)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Quỹ Đầu tư THS</v>
+      </c>
+      <c r="E35">
+        <v>10411000</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Chi trả cổ phần tháng 9</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>19:00:00 3/10/2026</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Mua sắm &amp; Tiêu dùng</v>
+      </c>
+      <c r="E36">
+        <v>500000</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Đi chợ</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>19:00:00 2/10/2026</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Ăn uống &amp; Cà phê</v>
+      </c>
+      <c r="E37">
+        <v>50000</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Mua đồ ăn vặt cho na ne</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
         <v>19:00:00 1/10/2026</v>
       </c>
-      <c r="C31" t="str">
-        <v>Thu nhập</v>
-      </c>
-      <c r="D31" t="str">
+      <c r="C38" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E38">
+        <v>90000</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Đổ xăng xe máy</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Chi tiêu</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Đi lại &amp; Xăng xe</v>
+      </c>
+      <c r="E39">
+        <v>280000</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Vé xe bus</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>19:00:00 1/10/2026</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Thu nhập</v>
+      </c>
+      <c r="D40" t="str">
         <v>Lương hàng tháng</v>
       </c>
-      <c r="E31">
+      <c r="E40">
         <v>18000000</v>
       </c>
-      <c r="F31" t="str">
-        <v>Tài khoản Ngân hàng (Chính)</v>
-      </c>
-      <c r="G31" t="str">
+      <c r="F40" t="str">
+        <v>Tài khoản Ngân hàng (Chính)</v>
+      </c>
+      <c r="G40" t="str">
         <v>lương tháng 10</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1246,7 +1453,7 @@
         <v>bank</v>
       </c>
       <c r="D2">
-        <v>30858000</v>
+        <v>32348000</v>
       </c>
     </row>
     <row r="3">

</xml_diff>